<commit_message>
Added a experiment run ultima template ingestion generic test. Tweaked the template to have it more similar to PacBio.
</commit_message>
<xml_diff>
--- a/backend/fms_core/static/submission_templates/Experiment_run_Ultima_v5_7_0.xlsx
+++ b/backend/fms_core/static/submission_templates/Experiment_run_Ultima_v5_7_0.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -8,10 +8,10 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Experiments" sheetId="1" state="visible" r:id="rId2"/>
-    <sheet name="Samples" sheetId="2" state="visible" r:id="rId3"/>
-    <sheet name="Info" sheetId="3" state="visible" r:id="rId4"/>
-    <sheet name="Index" sheetId="4" state="visible" r:id="rId5"/>
+    <sheet name="Experiments" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Samples" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Info" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Index" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="false" name="Ultima_wafer" vbProcedure="false">Index!$H$2</definedName>
@@ -38,7 +38,6 @@
             <sz val="10"/>
             <rFont val="Arial"/>
             <family val="2"/>
-            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">Illumina Flowcell Barcode</t>
         </r>
@@ -123,12 +122,12 @@
     <t xml:space="preserve">Comment</t>
   </si>
   <si>
+    <t xml:space="preserve">Sequencing Kit Lot</t>
+  </si>
+  <si>
     <t xml:space="preserve">Wafer Lot</t>
   </si>
   <si>
-    <t xml:space="preserve">Sequencing Kit Lot</t>
-  </si>
-  <si>
     <t xml:space="preserve">Sample Preparation</t>
   </si>
   <si>
@@ -201,15 +200,15 @@
     <t xml:space="preserve">Additional information related to the current experiment as a whole.</t>
   </si>
   <si>
+    <t xml:space="preserve">Sequencing kit lot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sequencing kit lot.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Wafer lot.</t>
   </si>
   <si>
-    <t xml:space="preserve">Sequencing kit lot</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sequencing kit lot.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Samples</t>
   </si>
   <si>
@@ -267,7 +266,7 @@
     <t xml:space="preserve">aDNA-ds</t>
   </si>
   <si>
-    <t xml:space="preserve">Krostie (V150)</t>
+    <t xml:space="preserve">Ultima UG100 (V150)</t>
   </si>
   <si>
     <t xml:space="preserve">Ultima wafer</t>
@@ -1594,7 +1593,6 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
@@ -1687,7 +1685,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -1730,6 +1728,13 @@
       <bottom style="thin"/>
       <diagonal/>
     </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -1756,7 +1761,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="33">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1813,10 +1818,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1869,15 +1870,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1889,15 +1882,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1991,13 +1984,119 @@
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
+  <a:themeElements>
+    <a:clrScheme name="LibreOffice">
+      <a:dk1>
+        <a:srgbClr val="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:srgbClr val="ffffff"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="000000"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="ffffff"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="18a303"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="0369a3"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="a33e03"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8e03a3"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="c99c00"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="c9211e"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000ee"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="551a8b"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme>
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:I996"/>
-  <sheetFormatPr defaultColWidth="14.515625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.51953125" defaultRowHeight="13.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="25.51"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="48.52"/>
@@ -2005,8 +2104,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="24.84"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="32.74"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="16.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="16.87"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="30.39"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="28.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="13.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="13.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="13"/>
@@ -2024,7 +2123,7 @@
       <c r="F1" s="3"/>
       <c r="G1" s="3"/>
     </row>
-    <row r="2" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
@@ -2129,7 +2228,7 @@
       <c r="F7" s="3"/>
       <c r="G7" s="13"/>
       <c r="H7" s="3"/>
-      <c r="I7" s="14"/>
+      <c r="I7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3"/>
@@ -2143,7 +2242,7 @@
       <c r="F8" s="3"/>
       <c r="G8" s="13"/>
       <c r="H8" s="3"/>
-      <c r="I8" s="14"/>
+      <c r="I8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3"/>
@@ -2157,7 +2256,7 @@
       <c r="F9" s="3"/>
       <c r="G9" s="13"/>
       <c r="H9" s="3"/>
-      <c r="I9" s="14"/>
+      <c r="I9" s="3"/>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3"/>
@@ -2171,7 +2270,7 @@
       <c r="F10" s="3"/>
       <c r="G10" s="13"/>
       <c r="H10" s="3"/>
-      <c r="I10" s="14"/>
+      <c r="I10" s="3"/>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3"/>
@@ -2185,7 +2284,7 @@
       <c r="F11" s="3"/>
       <c r="G11" s="13"/>
       <c r="H11" s="3"/>
-      <c r="I11" s="14"/>
+      <c r="I11" s="3"/>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3"/>
@@ -2199,7 +2298,7 @@
       <c r="F12" s="3"/>
       <c r="G12" s="13"/>
       <c r="H12" s="3"/>
-      <c r="I12" s="14"/>
+      <c r="I12" s="3"/>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3"/>
@@ -2213,7 +2312,7 @@
       <c r="F13" s="3"/>
       <c r="G13" s="13"/>
       <c r="H13" s="3"/>
-      <c r="I13" s="14"/>
+      <c r="I13" s="3"/>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3"/>
@@ -2227,7 +2326,7 @@
       <c r="F14" s="3"/>
       <c r="G14" s="13"/>
       <c r="H14" s="3"/>
-      <c r="I14" s="14"/>
+      <c r="I14" s="3"/>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3"/>
@@ -2241,7 +2340,7 @@
       <c r="F15" s="3"/>
       <c r="G15" s="13"/>
       <c r="H15" s="3"/>
-      <c r="I15" s="14"/>
+      <c r="I15" s="3"/>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3"/>
@@ -2255,7 +2354,7 @@
       <c r="F16" s="3"/>
       <c r="G16" s="13"/>
       <c r="H16" s="3"/>
-      <c r="I16" s="14"/>
+      <c r="I16" s="3"/>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="3"/>
@@ -2269,7 +2368,7 @@
       <c r="F17" s="3"/>
       <c r="G17" s="13"/>
       <c r="H17" s="3"/>
-      <c r="I17" s="14"/>
+      <c r="I17" s="3"/>
     </row>
     <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="3"/>
@@ -2283,7 +2382,7 @@
       <c r="F18" s="3"/>
       <c r="G18" s="13"/>
       <c r="H18" s="3"/>
-      <c r="I18" s="14"/>
+      <c r="I18" s="3"/>
     </row>
     <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="3"/>
@@ -2297,7 +2396,7 @@
       <c r="F19" s="3"/>
       <c r="G19" s="13"/>
       <c r="H19" s="3"/>
-      <c r="I19" s="14"/>
+      <c r="I19" s="3"/>
     </row>
     <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="3"/>
@@ -2311,7 +2410,7 @@
       <c r="F20" s="3"/>
       <c r="G20" s="13"/>
       <c r="H20" s="3"/>
-      <c r="I20" s="14"/>
+      <c r="I20" s="3"/>
     </row>
     <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="3"/>
@@ -2325,7 +2424,7 @@
       <c r="F21" s="3"/>
       <c r="G21" s="13"/>
       <c r="H21" s="3"/>
-      <c r="I21" s="14"/>
+      <c r="I21" s="3"/>
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="3"/>
@@ -2339,7 +2438,7 @@
       <c r="F22" s="3"/>
       <c r="G22" s="13"/>
       <c r="H22" s="3"/>
-      <c r="I22" s="14"/>
+      <c r="I22" s="3"/>
     </row>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="3"/>
@@ -2353,7 +2452,7 @@
       <c r="F23" s="3"/>
       <c r="G23" s="13"/>
       <c r="H23" s="3"/>
-      <c r="I23" s="14"/>
+      <c r="I23" s="3"/>
     </row>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="3"/>
@@ -2367,7 +2466,7 @@
       <c r="F24" s="3"/>
       <c r="G24" s="13"/>
       <c r="H24" s="3"/>
-      <c r="I24" s="14"/>
+      <c r="I24" s="3"/>
     </row>
     <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="3"/>
@@ -2381,7 +2480,7 @@
       <c r="F25" s="3"/>
       <c r="G25" s="13"/>
       <c r="H25" s="3"/>
-      <c r="I25" s="14"/>
+      <c r="I25" s="3"/>
     </row>
     <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="3"/>
@@ -2395,7 +2494,7 @@
       <c r="F26" s="3"/>
       <c r="G26" s="13"/>
       <c r="H26" s="3"/>
-      <c r="I26" s="14"/>
+      <c r="I26" s="3"/>
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="3"/>
@@ -2409,7 +2508,7 @@
       <c r="F27" s="3"/>
       <c r="G27" s="13"/>
       <c r="H27" s="3"/>
-      <c r="I27" s="14"/>
+      <c r="I27" s="3"/>
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="3"/>
@@ -2423,7 +2522,7 @@
       <c r="F28" s="3"/>
       <c r="G28" s="13"/>
       <c r="H28" s="3"/>
-      <c r="I28" s="14"/>
+      <c r="I28" s="3"/>
     </row>
     <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="3"/>
@@ -2437,7 +2536,7 @@
       <c r="F29" s="3"/>
       <c r="G29" s="13"/>
       <c r="H29" s="3"/>
-      <c r="I29" s="14"/>
+      <c r="I29" s="3"/>
     </row>
     <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="3"/>
@@ -2451,7 +2550,7 @@
       <c r="F30" s="3"/>
       <c r="G30" s="13"/>
       <c r="H30" s="3"/>
-      <c r="I30" s="14"/>
+      <c r="I30" s="3"/>
     </row>
     <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="3"/>
@@ -2465,7 +2564,7 @@
       <c r="F31" s="3"/>
       <c r="G31" s="13"/>
       <c r="H31" s="3"/>
-      <c r="I31" s="14"/>
+      <c r="I31" s="3"/>
     </row>
     <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="3"/>
@@ -2479,7 +2578,7 @@
       <c r="F32" s="3"/>
       <c r="G32" s="13"/>
       <c r="H32" s="3"/>
-      <c r="I32" s="14"/>
+      <c r="I32" s="3"/>
     </row>
     <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="3"/>
@@ -2493,7 +2592,7 @@
       <c r="F33" s="3"/>
       <c r="G33" s="13"/>
       <c r="H33" s="3"/>
-      <c r="I33" s="14"/>
+      <c r="I33" s="3"/>
     </row>
     <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="3"/>
@@ -2507,7 +2606,7 @@
       <c r="F34" s="3"/>
       <c r="G34" s="13"/>
       <c r="H34" s="3"/>
-      <c r="I34" s="14"/>
+      <c r="I34" s="3"/>
     </row>
     <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="3"/>
@@ -2521,7 +2620,7 @@
       <c r="F35" s="3"/>
       <c r="G35" s="13"/>
       <c r="H35" s="3"/>
-      <c r="I35" s="14"/>
+      <c r="I35" s="3"/>
     </row>
     <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="3"/>
@@ -2535,7 +2634,7 @@
       <c r="F36" s="3"/>
       <c r="G36" s="13"/>
       <c r="H36" s="3"/>
-      <c r="I36" s="14"/>
+      <c r="I36" s="3"/>
     </row>
     <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="3"/>
@@ -2549,7 +2648,7 @@
       <c r="F37" s="3"/>
       <c r="G37" s="13"/>
       <c r="H37" s="3"/>
-      <c r="I37" s="14"/>
+      <c r="I37" s="3"/>
     </row>
     <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="3"/>
@@ -2563,7 +2662,7 @@
       <c r="F38" s="3"/>
       <c r="G38" s="13"/>
       <c r="H38" s="3"/>
-      <c r="I38" s="14"/>
+      <c r="I38" s="3"/>
     </row>
     <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="3"/>
@@ -2577,7 +2676,7 @@
       <c r="F39" s="3"/>
       <c r="G39" s="13"/>
       <c r="H39" s="3"/>
-      <c r="I39" s="14"/>
+      <c r="I39" s="3"/>
     </row>
     <row r="40" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="3"/>
@@ -2591,7 +2690,7 @@
       <c r="F40" s="3"/>
       <c r="G40" s="13"/>
       <c r="H40" s="3"/>
-      <c r="I40" s="14"/>
+      <c r="I40" s="3"/>
     </row>
     <row r="41" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="3"/>
@@ -2605,7 +2704,7 @@
       <c r="F41" s="3"/>
       <c r="G41" s="13"/>
       <c r="H41" s="3"/>
-      <c r="I41" s="14"/>
+      <c r="I41" s="3"/>
     </row>
     <row r="42" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="3"/>
@@ -2619,7 +2718,7 @@
       <c r="F42" s="3"/>
       <c r="G42" s="13"/>
       <c r="H42" s="3"/>
-      <c r="I42" s="14"/>
+      <c r="I42" s="3"/>
     </row>
     <row r="43" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="3"/>
@@ -2633,7 +2732,7 @@
       <c r="F43" s="3"/>
       <c r="G43" s="13"/>
       <c r="H43" s="3"/>
-      <c r="I43" s="14"/>
+      <c r="I43" s="3"/>
     </row>
     <row r="44" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="3"/>
@@ -2647,7 +2746,7 @@
       <c r="F44" s="3"/>
       <c r="G44" s="13"/>
       <c r="H44" s="3"/>
-      <c r="I44" s="14"/>
+      <c r="I44" s="3"/>
     </row>
     <row r="45" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="3"/>
@@ -2661,7 +2760,7 @@
       <c r="F45" s="3"/>
       <c r="G45" s="13"/>
       <c r="H45" s="3"/>
-      <c r="I45" s="14"/>
+      <c r="I45" s="3"/>
     </row>
     <row r="46" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="3"/>
@@ -2675,7 +2774,7 @@
       <c r="F46" s="3"/>
       <c r="G46" s="13"/>
       <c r="H46" s="3"/>
-      <c r="I46" s="14"/>
+      <c r="I46" s="3"/>
     </row>
     <row r="47" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="3"/>
@@ -2689,7 +2788,7 @@
       <c r="F47" s="3"/>
       <c r="G47" s="13"/>
       <c r="H47" s="3"/>
-      <c r="I47" s="14"/>
+      <c r="I47" s="3"/>
     </row>
     <row r="48" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="3"/>
@@ -2703,7 +2802,7 @@
       <c r="F48" s="3"/>
       <c r="G48" s="13"/>
       <c r="H48" s="3"/>
-      <c r="I48" s="14"/>
+      <c r="I48" s="3"/>
     </row>
     <row r="49" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="3"/>
@@ -2717,7 +2816,7 @@
       <c r="F49" s="3"/>
       <c r="G49" s="13"/>
       <c r="H49" s="3"/>
-      <c r="I49" s="14"/>
+      <c r="I49" s="3"/>
     </row>
     <row r="50" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="3"/>
@@ -2731,7 +2830,7 @@
       <c r="F50" s="3"/>
       <c r="G50" s="13"/>
       <c r="H50" s="3"/>
-      <c r="I50" s="14"/>
+      <c r="I50" s="3"/>
     </row>
     <row r="51" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="3"/>
@@ -2745,7 +2844,7 @@
       <c r="F51" s="3"/>
       <c r="G51" s="13"/>
       <c r="H51" s="3"/>
-      <c r="I51" s="14"/>
+      <c r="I51" s="3"/>
     </row>
     <row r="52" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="3"/>
@@ -2759,7 +2858,7 @@
       <c r="F52" s="3"/>
       <c r="G52" s="13"/>
       <c r="H52" s="3"/>
-      <c r="I52" s="14"/>
+      <c r="I52" s="3"/>
     </row>
     <row r="53" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="3"/>
@@ -2773,7 +2872,7 @@
       <c r="F53" s="3"/>
       <c r="G53" s="13"/>
       <c r="H53" s="3"/>
-      <c r="I53" s="14"/>
+      <c r="I53" s="3"/>
     </row>
     <row r="54" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="3"/>
@@ -2787,7 +2886,7 @@
       <c r="F54" s="3"/>
       <c r="G54" s="13"/>
       <c r="H54" s="3"/>
-      <c r="I54" s="14"/>
+      <c r="I54" s="3"/>
     </row>
     <row r="55" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="3"/>
@@ -2801,7 +2900,7 @@
       <c r="F55" s="3"/>
       <c r="G55" s="13"/>
       <c r="H55" s="3"/>
-      <c r="I55" s="14"/>
+      <c r="I55" s="3"/>
     </row>
     <row r="56" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="3"/>
@@ -2815,7 +2914,7 @@
       <c r="F56" s="3"/>
       <c r="G56" s="13"/>
       <c r="H56" s="3"/>
-      <c r="I56" s="14"/>
+      <c r="I56" s="3"/>
     </row>
     <row r="57" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="3"/>
@@ -2829,7 +2928,7 @@
       <c r="F57" s="3"/>
       <c r="G57" s="13"/>
       <c r="H57" s="3"/>
-      <c r="I57" s="14"/>
+      <c r="I57" s="3"/>
     </row>
     <row r="58" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="3"/>
@@ -2843,7 +2942,7 @@
       <c r="F58" s="3"/>
       <c r="G58" s="13"/>
       <c r="H58" s="3"/>
-      <c r="I58" s="14"/>
+      <c r="I58" s="3"/>
     </row>
     <row r="59" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="3"/>
@@ -2857,7 +2956,7 @@
       <c r="F59" s="3"/>
       <c r="G59" s="13"/>
       <c r="H59" s="3"/>
-      <c r="I59" s="14"/>
+      <c r="I59" s="3"/>
     </row>
     <row r="60" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="3"/>
@@ -2871,7 +2970,7 @@
       <c r="F60" s="3"/>
       <c r="G60" s="13"/>
       <c r="H60" s="3"/>
-      <c r="I60" s="14"/>
+      <c r="I60" s="3"/>
     </row>
     <row r="61" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="3"/>
@@ -2885,7 +2984,7 @@
       <c r="F61" s="3"/>
       <c r="G61" s="13"/>
       <c r="H61" s="3"/>
-      <c r="I61" s="14"/>
+      <c r="I61" s="3"/>
     </row>
     <row r="62" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="3"/>
@@ -2899,7 +2998,7 @@
       <c r="F62" s="3"/>
       <c r="G62" s="13"/>
       <c r="H62" s="3"/>
-      <c r="I62" s="14"/>
+      <c r="I62" s="3"/>
     </row>
     <row r="63" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="3"/>
@@ -2913,7 +3012,7 @@
       <c r="F63" s="3"/>
       <c r="G63" s="13"/>
       <c r="H63" s="3"/>
-      <c r="I63" s="14"/>
+      <c r="I63" s="3"/>
     </row>
     <row r="64" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="3"/>
@@ -2927,7 +3026,7 @@
       <c r="F64" s="3"/>
       <c r="G64" s="13"/>
       <c r="H64" s="3"/>
-      <c r="I64" s="14"/>
+      <c r="I64" s="3"/>
     </row>
     <row r="65" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="3"/>
@@ -2941,7 +3040,7 @@
       <c r="F65" s="3"/>
       <c r="G65" s="13"/>
       <c r="H65" s="3"/>
-      <c r="I65" s="14"/>
+      <c r="I65" s="3"/>
     </row>
     <row r="66" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="3"/>
@@ -2955,7 +3054,7 @@
       <c r="F66" s="3"/>
       <c r="G66" s="13"/>
       <c r="H66" s="3"/>
-      <c r="I66" s="14"/>
+      <c r="I66" s="3"/>
     </row>
     <row r="67" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="3"/>
@@ -2969,7 +3068,7 @@
       <c r="F67" s="3"/>
       <c r="G67" s="13"/>
       <c r="H67" s="3"/>
-      <c r="I67" s="14"/>
+      <c r="I67" s="3"/>
     </row>
     <row r="68" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="3"/>
@@ -2983,7 +3082,7 @@
       <c r="F68" s="3"/>
       <c r="G68" s="13"/>
       <c r="H68" s="3"/>
-      <c r="I68" s="14"/>
+      <c r="I68" s="3"/>
     </row>
     <row r="69" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="3"/>
@@ -2997,7 +3096,7 @@
       <c r="F69" s="3"/>
       <c r="G69" s="13"/>
       <c r="H69" s="3"/>
-      <c r="I69" s="14"/>
+      <c r="I69" s="3"/>
     </row>
     <row r="70" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="3"/>
@@ -3011,7 +3110,7 @@
       <c r="F70" s="3"/>
       <c r="G70" s="13"/>
       <c r="H70" s="3"/>
-      <c r="I70" s="14"/>
+      <c r="I70" s="3"/>
     </row>
     <row r="71" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="3"/>
@@ -3025,7 +3124,7 @@
       <c r="F71" s="3"/>
       <c r="G71" s="13"/>
       <c r="H71" s="3"/>
-      <c r="I71" s="14"/>
+      <c r="I71" s="3"/>
     </row>
     <row r="72" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="3"/>
@@ -3039,7 +3138,7 @@
       <c r="F72" s="3"/>
       <c r="G72" s="13"/>
       <c r="H72" s="3"/>
-      <c r="I72" s="14"/>
+      <c r="I72" s="3"/>
     </row>
     <row r="73" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="3"/>
@@ -3053,7 +3152,7 @@
       <c r="F73" s="3"/>
       <c r="G73" s="13"/>
       <c r="H73" s="3"/>
-      <c r="I73" s="14"/>
+      <c r="I73" s="3"/>
     </row>
     <row r="74" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="3"/>
@@ -3067,7 +3166,7 @@
       <c r="F74" s="3"/>
       <c r="G74" s="13"/>
       <c r="H74" s="3"/>
-      <c r="I74" s="14"/>
+      <c r="I74" s="3"/>
     </row>
     <row r="75" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="3"/>
@@ -3081,7 +3180,7 @@
       <c r="F75" s="3"/>
       <c r="G75" s="13"/>
       <c r="H75" s="3"/>
-      <c r="I75" s="14"/>
+      <c r="I75" s="3"/>
     </row>
     <row r="76" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="3"/>
@@ -3095,7 +3194,7 @@
       <c r="F76" s="3"/>
       <c r="G76" s="13"/>
       <c r="H76" s="3"/>
-      <c r="I76" s="14"/>
+      <c r="I76" s="3"/>
     </row>
     <row r="77" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="3"/>
@@ -3109,7 +3208,7 @@
       <c r="F77" s="3"/>
       <c r="G77" s="13"/>
       <c r="H77" s="3"/>
-      <c r="I77" s="14"/>
+      <c r="I77" s="3"/>
     </row>
     <row r="78" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="3"/>
@@ -3123,7 +3222,7 @@
       <c r="F78" s="3"/>
       <c r="G78" s="13"/>
       <c r="H78" s="3"/>
-      <c r="I78" s="14"/>
+      <c r="I78" s="3"/>
     </row>
     <row r="79" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="3"/>
@@ -3137,7 +3236,7 @@
       <c r="F79" s="3"/>
       <c r="G79" s="13"/>
       <c r="H79" s="3"/>
-      <c r="I79" s="14"/>
+      <c r="I79" s="3"/>
     </row>
     <row r="80" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="3"/>
@@ -3151,7 +3250,7 @@
       <c r="F80" s="3"/>
       <c r="G80" s="13"/>
       <c r="H80" s="3"/>
-      <c r="I80" s="14"/>
+      <c r="I80" s="3"/>
     </row>
     <row r="81" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="3"/>
@@ -3165,7 +3264,7 @@
       <c r="F81" s="3"/>
       <c r="G81" s="13"/>
       <c r="H81" s="3"/>
-      <c r="I81" s="14"/>
+      <c r="I81" s="3"/>
     </row>
     <row r="82" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="3"/>
@@ -3179,7 +3278,7 @@
       <c r="F82" s="3"/>
       <c r="G82" s="13"/>
       <c r="H82" s="3"/>
-      <c r="I82" s="14"/>
+      <c r="I82" s="3"/>
     </row>
     <row r="83" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="3"/>
@@ -3193,7 +3292,7 @@
       <c r="F83" s="3"/>
       <c r="G83" s="13"/>
       <c r="H83" s="3"/>
-      <c r="I83" s="14"/>
+      <c r="I83" s="3"/>
     </row>
     <row r="84" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="3"/>
@@ -3207,7 +3306,7 @@
       <c r="F84" s="3"/>
       <c r="G84" s="13"/>
       <c r="H84" s="3"/>
-      <c r="I84" s="14"/>
+      <c r="I84" s="3"/>
     </row>
     <row r="85" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="3"/>
@@ -3221,7 +3320,7 @@
       <c r="F85" s="3"/>
       <c r="G85" s="13"/>
       <c r="H85" s="3"/>
-      <c r="I85" s="14"/>
+      <c r="I85" s="3"/>
     </row>
     <row r="86" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="3"/>
@@ -3235,7 +3334,7 @@
       <c r="F86" s="3"/>
       <c r="G86" s="13"/>
       <c r="H86" s="3"/>
-      <c r="I86" s="14"/>
+      <c r="I86" s="3"/>
     </row>
     <row r="87" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="3"/>
@@ -3249,7 +3348,7 @@
       <c r="F87" s="3"/>
       <c r="G87" s="13"/>
       <c r="H87" s="3"/>
-      <c r="I87" s="14"/>
+      <c r="I87" s="3"/>
     </row>
     <row r="88" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="3"/>
@@ -3263,7 +3362,7 @@
       <c r="F88" s="3"/>
       <c r="G88" s="13"/>
       <c r="H88" s="3"/>
-      <c r="I88" s="14"/>
+      <c r="I88" s="3"/>
     </row>
     <row r="89" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A89" s="3"/>
@@ -3277,7 +3376,7 @@
       <c r="F89" s="3"/>
       <c r="G89" s="13"/>
       <c r="H89" s="3"/>
-      <c r="I89" s="14"/>
+      <c r="I89" s="3"/>
     </row>
     <row r="90" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="3"/>
@@ -3291,7 +3390,7 @@
       <c r="F90" s="3"/>
       <c r="G90" s="13"/>
       <c r="H90" s="3"/>
-      <c r="I90" s="14"/>
+      <c r="I90" s="3"/>
     </row>
     <row r="91" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="3"/>
@@ -3305,7 +3404,7 @@
       <c r="F91" s="3"/>
       <c r="G91" s="13"/>
       <c r="H91" s="3"/>
-      <c r="I91" s="14"/>
+      <c r="I91" s="3"/>
     </row>
     <row r="92" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A92" s="3"/>
@@ -3319,7 +3418,7 @@
       <c r="F92" s="3"/>
       <c r="G92" s="13"/>
       <c r="H92" s="3"/>
-      <c r="I92" s="14"/>
+      <c r="I92" s="3"/>
     </row>
     <row r="93" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A93" s="3"/>
@@ -3333,7 +3432,7 @@
       <c r="F93" s="3"/>
       <c r="G93" s="13"/>
       <c r="H93" s="3"/>
-      <c r="I93" s="14"/>
+      <c r="I93" s="3"/>
     </row>
     <row r="94" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A94" s="3"/>
@@ -3347,7 +3446,7 @@
       <c r="F94" s="3"/>
       <c r="G94" s="13"/>
       <c r="H94" s="3"/>
-      <c r="I94" s="14"/>
+      <c r="I94" s="3"/>
     </row>
     <row r="95" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A95" s="3"/>
@@ -3361,7 +3460,7 @@
       <c r="F95" s="3"/>
       <c r="G95" s="13"/>
       <c r="H95" s="3"/>
-      <c r="I95" s="14"/>
+      <c r="I95" s="3"/>
     </row>
     <row r="96" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A96" s="3"/>
@@ -3375,7 +3474,7 @@
       <c r="F96" s="3"/>
       <c r="G96" s="13"/>
       <c r="H96" s="3"/>
-      <c r="I96" s="14"/>
+      <c r="I96" s="3"/>
     </row>
     <row r="97" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A97" s="3"/>
@@ -3389,7 +3488,7 @@
       <c r="F97" s="13"/>
       <c r="G97" s="13"/>
       <c r="H97" s="3"/>
-      <c r="I97" s="14"/>
+      <c r="I97" s="3"/>
     </row>
     <row r="98" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A98" s="3"/>
@@ -3403,7 +3502,7 @@
       <c r="F98" s="13"/>
       <c r="G98" s="13"/>
       <c r="H98" s="3"/>
-      <c r="I98" s="14"/>
+      <c r="I98" s="3"/>
     </row>
     <row r="99" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A99" s="3"/>
@@ -3417,7 +3516,7 @@
       <c r="F99" s="13"/>
       <c r="G99" s="13"/>
       <c r="H99" s="3"/>
-      <c r="I99" s="14"/>
+      <c r="I99" s="3"/>
     </row>
     <row r="100" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A100" s="3"/>
@@ -3431,7 +3530,7 @@
       <c r="F100" s="13"/>
       <c r="G100" s="13"/>
       <c r="H100" s="3"/>
-      <c r="I100" s="14"/>
+      <c r="I100" s="3"/>
     </row>
     <row r="101" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A101" s="3"/>
@@ -5264,22 +5363,22 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D7:D100" type="list">
-      <formula1>Index!$F$2:$F$2</formula1>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D7:D100" type="list">
+      <formula1>Index!$F$2</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="E8:E100" type="list">
-      <formula1>INDIRECT(SUBSTITUTE(INDEX(Index!$G$2:$G$2, MATCH(C7, Index!$F$2:$F$2, 0), 1), " ", "_"))</formula1>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="E8:E100" type="list">
+      <formula1>INDIRECT(SUBSTITUTE(INDEX(Index!$G$2, MATCH(C7, Index!$F$2, 0), 1), " ", "_"))</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="E7" type="list">
-      <formula1>INDIRECT(SUBSTITUTE(INDEX(Index!$G$2:$G$2, MATCH(D7, Index!$F$2:$F$2, 0), 1), " ", "_"))</formula1>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="E7" type="list">
+      <formula1>INDIRECT(SUBSTITUTE(INDEX(Index!$G$2, MATCH(D7, Index!$F$2, 0), 1), " ", "_"))</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
-  <pageSetup paperSize="1" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -5289,23 +5388,23 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:K1000"/>
-  <sheetFormatPr defaultColWidth="14.515625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.51953125" defaultRowHeight="13.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="1" style="1" width="24.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="25.84"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="30.64"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="32.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="34.16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="36.94"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="47.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="24.6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="13.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="1024" style="0" width="9.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="27.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="41.55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="1024" style="1" width="9.14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5340,21 +5439,21 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="15" t="s">
+      <c r="A3" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="15"/>
+      <c r="B3" s="14"/>
       <c r="C3" s="9"/>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
-      <c r="F3" s="16"/>
+      <c r="F3" s="15"/>
       <c r="G3" s="9"/>
       <c r="H3" s="9"/>
       <c r="I3" s="9"/>
-      <c r="J3" s="17" t="s">
+      <c r="J3" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="K3" s="17"/>
+      <c r="K3" s="16"/>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
@@ -5381,7 +5480,7 @@
       <c r="H4" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="I4" s="18" t="s">
+      <c r="I4" s="17" t="s">
         <v>24</v>
       </c>
       <c r="J4" s="11" t="s">
@@ -5400,7 +5499,6 @@
       <c r="G5" s="3"/>
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
-      <c r="J5" s="0"/>
       <c r="K5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5412,7 +5510,6 @@
       <c r="G6" s="3"/>
       <c r="H6" s="3"/>
       <c r="I6" s="3"/>
-      <c r="J6" s="0"/>
       <c r="K6" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5551,8 +5648,8 @@
       <c r="A19" s="3"/>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
-      <c r="D19" s="19"/>
-      <c r="E19" s="19"/>
+      <c r="D19" s="18"/>
+      <c r="E19" s="18"/>
       <c r="G19" s="3"/>
       <c r="H19" s="3"/>
       <c r="I19" s="3"/>
@@ -9754,34 +9851,34 @@
     <mergeCell ref="J3:K3"/>
   </mergeCells>
   <dataValidations count="6">
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D5:D101" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D5:D101" type="list">
       <formula1>Index!$B$2:$B$97</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="A5:A100" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="A5:A100" type="list">
       <formula1>Experiments!$A$7:$A$106</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="I5:I100" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="I5:I100" type="list">
       <formula1>Index!$D$2:$D$5</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="E5:E101" type="none">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="E5:E101" type="none">
       <formula1>Index!$B$2:$B$97</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G5:G1000" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G5:G1000" type="list">
       <formula1>Index!$A$2:$A$9</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="K5:K100" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="K5:K100" type="list">
       <formula1>Index!$E$2:$E$32</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
-  <pageSetup paperSize="1" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -9790,24 +9887,24 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C31"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.18359375" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="45.68"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="19" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="21" t="s">
+      <c r="A3" s="20" t="s">
         <v>28</v>
       </c>
     </row>
@@ -9823,214 +9920,212 @@
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="7" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="22" t="s">
+      <c r="A7" s="21" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="21"/>
-      <c r="B8" s="23"/>
+      <c r="A8" s="20"/>
+      <c r="B8" s="22"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="24" t="s">
+      <c r="A9" s="23" t="s">
         <v>32</v>
       </c>
-      <c r="B9" s="23"/>
+      <c r="B9" s="22"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="25" t="s">
+      <c r="A10" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="26" t="s">
+      <c r="B10" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="C10" s="27"/>
+      <c r="C10" s="26"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="25" t="s">
+      <c r="A11" s="24" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="26" t="s">
+      <c r="B11" s="25" t="s">
         <v>34</v>
       </c>
-      <c r="C11" s="27"/>
+      <c r="C11" s="26"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="28" t="s">
+      <c r="A12" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="B12" s="29" t="s">
+      <c r="B12" s="25" t="s">
         <v>35</v>
       </c>
-      <c r="C12" s="27"/>
+      <c r="C12" s="26"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="25" t="s">
+      <c r="A13" s="24" t="s">
         <v>10</v>
       </c>
-      <c r="B13" s="26" t="s">
+      <c r="B13" s="25" t="s">
         <v>36</v>
       </c>
-      <c r="C13" s="27"/>
+      <c r="C13" s="26"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="23" t="s">
+      <c r="A14" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="26" t="s">
+      <c r="B14" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="C14" s="27"/>
+      <c r="C14" s="26"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="25" t="s">
+      <c r="A15" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="B15" s="26" t="s">
+      <c r="B15" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="C15" s="27"/>
+      <c r="C15" s="26"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="25" t="s">
+      <c r="A16" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="B16" s="26" t="s">
+      <c r="B16" s="25" t="s">
         <v>39</v>
       </c>
-      <c r="C16" s="27"/>
-    </row>
-    <row r="17" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="25" t="s">
-        <v>14</v>
-      </c>
-      <c r="B17" s="30" t="s">
+      <c r="C16" s="26"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="24" t="s">
         <v>40</v>
       </c>
-      <c r="C17" s="27"/>
+      <c r="B17" s="25" t="s">
+        <v>41</v>
+      </c>
+      <c r="C17" s="26"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="25" t="s">
-        <v>41</v>
-      </c>
-      <c r="B18" s="26" t="s">
+      <c r="A18" s="24" t="s">
+        <v>15</v>
+      </c>
+      <c r="B18" s="27" t="s">
         <v>42</v>
       </c>
-      <c r="C18" s="27"/>
-    </row>
-    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0"/>
-    </row>
+      <c r="C18" s="26"/>
+    </row>
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="31" t="s">
+      <c r="A20" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="B20" s="32"/>
-      <c r="C20" s="32"/>
+      <c r="B20" s="29"/>
+      <c r="C20" s="29"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="25" t="s">
+      <c r="A21" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="B21" s="26" t="s">
+      <c r="B21" s="25" t="s">
         <v>44</v>
       </c>
-      <c r="C21" s="27"/>
+      <c r="C21" s="26"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="25" t="s">
+      <c r="A22" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="B22" s="26" t="s">
+      <c r="B22" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="C22" s="27"/>
+      <c r="C22" s="26"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="25" t="s">
+      <c r="A23" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="B23" s="26" t="s">
+      <c r="B23" s="25" t="s">
         <v>46</v>
       </c>
-      <c r="C23" s="27"/>
+      <c r="C23" s="26"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="25" t="s">
+      <c r="A24" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="B24" s="26" t="s">
+      <c r="B24" s="25" t="s">
         <v>47</v>
       </c>
-      <c r="C24" s="27"/>
+      <c r="C24" s="26"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="25" t="s">
+      <c r="A25" s="24" t="s">
         <v>21</v>
       </c>
-      <c r="B25" s="26" t="s">
+      <c r="B25" s="25" t="s">
         <v>48</v>
       </c>
-      <c r="C25" s="27"/>
+      <c r="C25" s="26"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="25" t="s">
+      <c r="A26" s="24" t="s">
         <v>22</v>
       </c>
-      <c r="B26" s="26" t="s">
+      <c r="B26" s="25" t="s">
         <v>49</v>
       </c>
-      <c r="C26" s="27"/>
+      <c r="C26" s="26"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="25" t="s">
+      <c r="A27" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="B27" s="26" t="s">
+      <c r="B27" s="25" t="s">
         <v>50</v>
       </c>
-      <c r="C27" s="27"/>
+      <c r="C27" s="26"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="25" t="s">
+      <c r="A28" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="B28" s="26" t="s">
+      <c r="B28" s="25" t="s">
         <v>51</v>
       </c>
-      <c r="C28" s="27"/>
+      <c r="C28" s="26"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="25" t="s">
+      <c r="A29" s="24" t="s">
         <v>24</v>
       </c>
-      <c r="B29" s="26" t="s">
+      <c r="B29" s="25" t="s">
         <v>52</v>
       </c>
-      <c r="C29" s="27"/>
+      <c r="C29" s="26"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="25" t="s">
+      <c r="A30" s="24" t="s">
         <v>25</v>
       </c>
-      <c r="B30" s="26" t="s">
+      <c r="B30" s="25" t="s">
         <v>53</v>
       </c>
-      <c r="C30" s="27"/>
+      <c r="C30" s="26"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="25" t="s">
+      <c r="A31" s="24" t="s">
         <v>26</v>
       </c>
-      <c r="B31" s="26" t="s">
+      <c r="B31" s="25" t="s">
         <v>54</v>
       </c>
-      <c r="C31" s="27"/>
+      <c r="C31" s="26"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="1" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
@@ -10039,12 +10134,12 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H1000"/>
-  <sheetFormatPr defaultColWidth="14.515625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.51953125" defaultRowHeight="13.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16.5"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16.83"/>
@@ -10054,8 +10149,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="25.72"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="26.02"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="23.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1020" min="1019" style="1" width="9.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="1021" style="0" width="9.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="1019" style="1" width="9.14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10080,7 +10174,7 @@
       <c r="G1" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="H1" s="21" t="s">
+      <c r="H1" s="20" t="s">
         <v>11</v>
       </c>
     </row>
@@ -10097,13 +10191,13 @@
       <c r="D2" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="E2" s="33" t="s">
+      <c r="E2" s="30" t="s">
         <v>61</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="G2" s="21" t="s">
+      <c r="G2" s="20" t="s">
         <v>63</v>
       </c>
       <c r="H2" s="1" t="s">
@@ -10120,7 +10214,7 @@
       <c r="D3" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="E3" s="33" t="s">
+      <c r="E3" s="30" t="s">
         <v>66</v>
       </c>
     </row>
@@ -10134,7 +10228,7 @@
       <c r="D4" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="E4" s="34" t="s">
+      <c r="E4" s="31" t="s">
         <v>69</v>
       </c>
     </row>
@@ -10148,7 +10242,7 @@
       <c r="D5" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="E5" s="33" t="s">
+      <c r="E5" s="30" t="s">
         <v>72</v>
       </c>
     </row>
@@ -10159,7 +10253,7 @@
       <c r="C6" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="E6" s="33" t="s">
+      <c r="E6" s="30" t="s">
         <v>74</v>
       </c>
     </row>
@@ -10170,7 +10264,7 @@
       <c r="C7" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="E7" s="33" t="s">
+      <c r="E7" s="30" t="s">
         <v>76</v>
       </c>
     </row>
@@ -10181,7 +10275,7 @@
       <c r="C8" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="E8" s="33" t="s">
+      <c r="E8" s="30" t="s">
         <v>78</v>
       </c>
     </row>
@@ -10192,7 +10286,7 @@
       <c r="C9" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="E9" s="33" t="s">
+      <c r="E9" s="30" t="s">
         <v>80</v>
       </c>
     </row>
@@ -10203,7 +10297,7 @@
       <c r="C10" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="E10" s="33" t="s">
+      <c r="E10" s="30" t="s">
         <v>82</v>
       </c>
     </row>
@@ -10214,7 +10308,7 @@
       <c r="C11" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="E11" s="33" t="s">
+      <c r="E11" s="30" t="s">
         <v>84</v>
       </c>
     </row>
@@ -10225,7 +10319,7 @@
       <c r="C12" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="E12" s="33" t="s">
+      <c r="E12" s="30" t="s">
         <v>86</v>
       </c>
     </row>
@@ -10236,7 +10330,7 @@
       <c r="C13" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="E13" s="33" t="s">
+      <c r="E13" s="30" t="s">
         <v>88</v>
       </c>
     </row>
@@ -10247,7 +10341,7 @@
       <c r="C14" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="E14" s="33" t="s">
+      <c r="E14" s="30" t="s">
         <v>91</v>
       </c>
     </row>
@@ -10258,7 +10352,7 @@
       <c r="C15" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="E15" s="33" t="s">
+      <c r="E15" s="30" t="s">
         <v>94</v>
       </c>
     </row>
@@ -10269,7 +10363,7 @@
       <c r="C16" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="E16" s="33" t="s">
+      <c r="E16" s="30" t="s">
         <v>97</v>
       </c>
     </row>
@@ -10280,7 +10374,7 @@
       <c r="C17" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="E17" s="33" t="s">
+      <c r="E17" s="30" t="s">
         <v>100</v>
       </c>
     </row>
@@ -10291,7 +10385,7 @@
       <c r="C18" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="E18" s="33" t="s">
+      <c r="E18" s="30" t="s">
         <v>103</v>
       </c>
     </row>
@@ -10302,7 +10396,7 @@
       <c r="C19" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="E19" s="33" t="s">
+      <c r="E19" s="30" t="s">
         <v>106</v>
       </c>
     </row>
@@ -10313,7 +10407,7 @@
       <c r="C20" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="E20" s="33" t="s">
+      <c r="E20" s="30" t="s">
         <v>109</v>
       </c>
     </row>
@@ -10324,7 +10418,7 @@
       <c r="C21" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="E21" s="33" t="s">
+      <c r="E21" s="30" t="s">
         <v>112</v>
       </c>
     </row>
@@ -10335,7 +10429,7 @@
       <c r="C22" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="E22" s="33" t="s">
+      <c r="E22" s="30" t="s">
         <v>115</v>
       </c>
     </row>
@@ -10346,7 +10440,7 @@
       <c r="C23" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="E23" s="33" t="s">
+      <c r="E23" s="30" t="s">
         <v>118</v>
       </c>
     </row>
@@ -10357,7 +10451,7 @@
       <c r="C24" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="E24" s="33" t="s">
+      <c r="E24" s="30" t="s">
         <v>121</v>
       </c>
     </row>
@@ -10368,7 +10462,7 @@
       <c r="C25" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="E25" s="33" t="s">
+      <c r="E25" s="30" t="s">
         <v>124</v>
       </c>
     </row>
@@ -10379,7 +10473,7 @@
       <c r="C26" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="E26" s="33" t="s">
+      <c r="E26" s="30" t="s">
         <v>126</v>
       </c>
     </row>
@@ -10390,7 +10484,7 @@
       <c r="C27" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="E27" s="34" t="s">
+      <c r="E27" s="31" t="s">
         <v>128</v>
       </c>
     </row>
@@ -10401,7 +10495,7 @@
       <c r="C28" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="E28" s="34" t="s">
+      <c r="E28" s="31" t="s">
         <v>130</v>
       </c>
     </row>
@@ -10412,7 +10506,7 @@
       <c r="C29" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="E29" s="33" t="s">
+      <c r="E29" s="30" t="s">
         <v>132</v>
       </c>
     </row>
@@ -10423,7 +10517,7 @@
       <c r="C30" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="E30" s="33" t="s">
+      <c r="E30" s="30" t="s">
         <v>134</v>
       </c>
     </row>
@@ -10434,7 +10528,7 @@
       <c r="C31" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="E31" s="33" t="s">
+      <c r="E31" s="30" t="s">
         <v>136</v>
       </c>
     </row>
@@ -10445,7 +10539,7 @@
       <c r="C32" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="E32" s="35" t="s">
+      <c r="E32" s="32" t="s">
         <v>138</v>
       </c>
     </row>
@@ -13026,14 +13120,14 @@
     <row r="1000" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G2" type="none">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G2" type="none">
       <formula1>Index!$H$2</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0" footer="0"/>
-  <pageSetup paperSize="1" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;A</oddHeader>
     <oddFooter>&amp;CPage &amp;P</oddFooter>

</xml_diff>